<commit_message>
BOM changes for soldering
</commit_message>
<xml_diff>
--- a/BOM/BOM_Platine.xlsx
+++ b/BOM/BOM_Platine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Semester6\Projektarbeit\Projektarbeit_Joystick\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A1D378B-F9A9-4F9A-A819-BDFC437B318E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C675947-B90C-463C-A206-C034444DF022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00578EB7-767E-4B19-B43A-D2F6E31B5412}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="99">
   <si>
     <t>Bauteilgruppe</t>
   </si>
@@ -333,6 +333,9 @@
   </si>
   <si>
     <t>Widerstand R1</t>
+  </si>
+  <si>
+    <t>Slotnummer</t>
   </si>
 </sst>
 </file>
@@ -408,7 +411,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -451,11 +454,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -518,6 +532,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -852,7 +867,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F25D80F-7FB9-48DC-8DAC-13AD3380FE13}">
-  <dimension ref="B2:I35"/>
+  <dimension ref="B2:J35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="21.90625" bestFit="1" customWidth="1"/>
@@ -865,7 +880,7 @@
     <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B2" s="13" t="s">
         <v>0</v>
       </c>
@@ -890,8 +905,11 @@
       <c r="I2" s="13" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J2" s="34" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B3" s="27" t="s">
         <v>3</v>
       </c>
@@ -914,8 +932,11 @@
         <v>4</v>
       </c>
       <c r="I3" s="3"/>
-    </row>
-    <row r="4" spans="2:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="J3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" ht="29" x14ac:dyDescent="0.35">
       <c r="B4" s="27"/>
       <c r="C4" s="1" t="s">
         <v>6</v>
@@ -936,8 +957,11 @@
         <v>1</v>
       </c>
       <c r="I4" s="3"/>
-    </row>
-    <row r="5" spans="2:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="J4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" ht="29" x14ac:dyDescent="0.35">
       <c r="B5" s="27"/>
       <c r="C5" s="3" t="s">
         <v>6</v>
@@ -958,8 +982,11 @@
         <v>1</v>
       </c>
       <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B6" s="27"/>
       <c r="C6" s="3" t="s">
         <v>6</v>
@@ -980,8 +1007,11 @@
         <v>1</v>
       </c>
       <c r="I6" s="3"/>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J6">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B7" s="27"/>
       <c r="C7" s="3" t="s">
         <v>20</v>
@@ -1003,7 +1033,7 @@
       </c>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B8" s="27"/>
       <c r="C8" s="3" t="s">
         <v>21</v>
@@ -1025,7 +1055,7 @@
       </c>
       <c r="I8" s="3"/>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B9" s="27"/>
       <c r="C9" s="1" t="s">
         <v>24</v>
@@ -1047,7 +1077,7 @@
       </c>
       <c r="I9" s="3"/>
     </row>
-    <row r="10" spans="2:9" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:10" ht="29" x14ac:dyDescent="0.35">
       <c r="B10" s="27"/>
       <c r="C10" s="3" t="s">
         <v>27</v>
@@ -1069,7 +1099,7 @@
       </c>
       <c r="I10" s="3"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B11" s="27"/>
       <c r="C11" s="3" t="s">
         <v>31</v>
@@ -1090,8 +1120,11 @@
         <v>54</v>
       </c>
       <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B12" s="28" t="s">
         <v>34</v>
       </c>
@@ -1115,7 +1148,7 @@
       </c>
       <c r="I12" s="7"/>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B13" s="29"/>
       <c r="C13" s="7" t="s">
         <v>95</v>
@@ -1136,8 +1169,11 @@
         <v>3</v>
       </c>
       <c r="I13" s="7"/>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B14" s="29"/>
       <c r="C14" s="7" t="s">
         <v>39</v>
@@ -1159,7 +1195,7 @@
       </c>
       <c r="I14" s="7"/>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B15" s="29"/>
       <c r="C15" s="7" t="s">
         <v>97</v>
@@ -1180,8 +1216,11 @@
         <v>3</v>
       </c>
       <c r="I15" s="7"/>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B16" s="30"/>
       <c r="C16" s="7" t="s">
         <v>43</v>
@@ -1203,7 +1242,7 @@
       </c>
       <c r="I16" s="7"/>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B17" s="30"/>
       <c r="C17" s="7" t="s">
         <v>24</v>
@@ -1224,8 +1263,11 @@
         <v>2</v>
       </c>
       <c r="I17" s="7"/>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B18" s="31" t="s">
         <v>47</v>
       </c>
@@ -1246,8 +1288,11 @@
         <v>2</v>
       </c>
       <c r="I18" s="10"/>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J18">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B19" s="31"/>
       <c r="C19" s="10" t="s">
         <v>24</v>
@@ -1268,8 +1313,11 @@
         <v>2</v>
       </c>
       <c r="I19" s="10"/>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B20" s="30"/>
       <c r="C20" s="10" t="s">
         <v>6</v>
@@ -1291,7 +1339,7 @@
       </c>
       <c r="I20" s="10"/>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B21" s="32" t="s">
         <v>55</v>
       </c>
@@ -1315,7 +1363,7 @@
       </c>
       <c r="I21" s="15"/>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B22" s="32"/>
       <c r="C22" s="15" t="s">
         <v>74</v>
@@ -1337,7 +1385,7 @@
       </c>
       <c r="I22" s="15"/>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B23" s="32"/>
       <c r="C23" s="15" t="s">
         <v>24</v>
@@ -1358,8 +1406,11 @@
         <v>2</v>
       </c>
       <c r="I23" s="15"/>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B24" s="32"/>
       <c r="C24" s="15" t="s">
         <v>62</v>
@@ -1381,7 +1432,7 @@
       </c>
       <c r="I24" s="15"/>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B25" s="32"/>
       <c r="C25" s="15" t="s">
         <v>65</v>
@@ -1402,8 +1453,11 @@
         <v>1</v>
       </c>
       <c r="I25" s="15"/>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B26" s="32"/>
       <c r="C26" s="15" t="s">
         <v>69</v>
@@ -1425,7 +1479,7 @@
       </c>
       <c r="I26" s="15"/>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B27" s="33"/>
       <c r="C27" s="15" t="s">
         <v>71</v>
@@ -1447,7 +1501,7 @@
       </c>
       <c r="I27" s="15"/>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B28" s="33"/>
       <c r="C28" s="15" t="s">
         <v>73</v>
@@ -1469,7 +1523,7 @@
       </c>
       <c r="I28" s="15"/>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B29" s="33"/>
       <c r="C29" s="15" t="s">
         <v>73</v>
@@ -1490,8 +1544,11 @@
         <v>1</v>
       </c>
       <c r="I29" s="15"/>
-    </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J29">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B30" s="30"/>
       <c r="C30" s="15" t="s">
         <v>77</v>
@@ -1511,7 +1568,7 @@
       </c>
       <c r="I30" s="15"/>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B31" s="25" t="s">
         <v>80</v>
       </c>
@@ -1533,7 +1590,7 @@
       </c>
       <c r="I31" s="18"/>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B32" s="26"/>
       <c r="C32" s="18" t="s">
         <v>83</v>

</xml_diff>